<commit_message>
src011 update with h2 side fluorophore staples
</commit_message>
<xml_diff>
--- a/crisscross_kit/crisscross/dna_source_plates/assembly_plates/sw_src011_fluorescenthandles.xlsx
+++ b/crisscross_kit/crisscross/dna_source_plates/assembly_plates/sw_src011_fluorescenthandles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt/Documents/Shih_Lab_Postdoc/research_projects/crisscross_code/crisscross_kit/crisscross/dna_source_plates/assembly_plates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stellawang/Documents/gitrepos/Crisscross-Design/crisscross_kit/crisscross/dna_source_plates/assembly_plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6EB6047-F3EF-4D4D-84A7-C76E98E95A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA305B96-40A4-3E40-98BC-0F92CB9BEA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25600" yWindow="620" windowWidth="25600" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="454">
   <si>
     <t>well</t>
   </si>
@@ -1366,13 +1366,31 @@
   </si>
   <si>
     <t>ASSEMBLY_HANDLE_v2-58-h5-position_30</t>
+  </si>
+  <si>
+    <t>ASSEMBLY_ANTIHANDLE_v2-5-h2-position_26</t>
+  </si>
+  <si>
+    <t>atto532n</t>
+  </si>
+  <si>
+    <t>Fluorescent Assembly Antihandle For Slat Position 26, Handle 5, Fluorophore Atto532 Side h2, originally from SSW121</t>
+  </si>
+  <si>
+    <t>Fluorescent Assembly Antihandle For Slat Position 26, Handle 5, Fluorophore Atto647 Side h2, originally from SSW122</t>
+  </si>
+  <si>
+    <t>TATTTATCCCAAGCATTAGACGGGAGAATTATAAGAGCAAGAtt TCCACTA /3ATTO532N/</t>
+  </si>
+  <si>
+    <t>TATTTATCCCAAGCATTAGACGGGAGAATTATAAGAGCAAGAtt TCCACTA /3ATTO647N/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1387,12 +1405,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Helvetica"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1465,7 +1477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1473,11 +1485,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1811,7 +1820,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>443</v>
       </c>
     </row>
@@ -2669,7 +2678,7 @@
       <c r="A52" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="6" t="s">
+      <c r="B52" s="5" t="s">
         <v>445</v>
       </c>
       <c r="C52" t="s">
@@ -2689,7 +2698,7 @@
       <c r="A53" t="s">
         <v>56</v>
       </c>
-      <c r="B53" s="6" t="s">
+      <c r="B53" s="5" t="s">
         <v>446</v>
       </c>
       <c r="C53" t="s">
@@ -2709,7 +2718,7 @@
       <c r="A54" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="5" t="s">
         <v>447</v>
       </c>
       <c r="C54" t="s">
@@ -2882,15 +2891,11 @@
       <c r="A76" t="s">
         <v>79</v>
       </c>
-      <c r="B76" s="5"/>
-      <c r="C76" s="6"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>80</v>
       </c>
-      <c r="B77" s="5"/>
-      <c r="C77" s="6"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
@@ -3671,7 +3676,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>196</v>
       </c>
@@ -3688,7 +3693,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>197</v>
       </c>
@@ -3705,7 +3710,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>198</v>
       </c>
@@ -3722,67 +3727,97 @@
         <v>100</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B196" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="C196" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="D196" t="s">
+        <v>450</v>
+      </c>
+      <c r="E196">
+        <v>100</v>
+      </c>
+      <c r="F196" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B197" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="C197" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D197" t="s">
+        <v>451</v>
+      </c>
+      <c r="E197">
+        <v>100</v>
+      </c>
+      <c r="F197" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>211</v>
       </c>
@@ -5607,775 +5642,777 @@
       <c r="A2" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="P2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Q2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="S2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="T2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="U2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="W2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="X2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y2" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z2" s="6"/>
+      <c r="B2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z2" s="5"/>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="T3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="V3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="W3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="X3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y3" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z3" s="6"/>
+      <c r="B3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z3" s="5"/>
     </row>
     <row r="4" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>432</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>434</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-      <c r="X4" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y4" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z4" s="6"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z4" s="5"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
-      <c r="T5" s="6"/>
-      <c r="U5" s="6"/>
-      <c r="V5" s="6"/>
-      <c r="W5" s="6"/>
-      <c r="X5" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y5" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z5" s="6"/>
+      <c r="B5" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="5"/>
+      <c r="W5" s="5"/>
+      <c r="X5" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z5" s="5"/>
     </row>
     <row r="6" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="6"/>
-      <c r="W6" s="6"/>
-      <c r="X6" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y6" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z6" s="6"/>
+      <c r="B6" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z6" s="5"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-      <c r="T7" s="6"/>
-      <c r="U7" s="6"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y7" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z7" s="6"/>
+      <c r="B7" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y7" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z7" s="5"/>
     </row>
     <row r="8" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="6"/>
-      <c r="W8" s="6"/>
-      <c r="X8" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y8" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z8" s="6"/>
+      <c r="B8" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="5"/>
+      <c r="X8" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y8" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z8" s="5"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
-      <c r="X9" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y9" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z9" s="6"/>
+      <c r="B9" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+      <c r="X9" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z9" s="5"/>
     </row>
     <row r="10" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="6"/>
-      <c r="X10" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y10" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z10" s="6"/>
+      <c r="B10" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+      <c r="X10" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z10" s="5"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="6"/>
-      <c r="X11" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y11" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z11" s="6"/>
+      <c r="B11" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="5"/>
+      <c r="W11" s="5"/>
+      <c r="X11" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z11" s="5"/>
     </row>
     <row r="12" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="6"/>
-      <c r="W12" s="6"/>
-      <c r="X12" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y12" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z12" s="6"/>
+      <c r="B12" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="5"/>
+      <c r="T12" s="5"/>
+      <c r="U12" s="5"/>
+      <c r="V12" s="5"/>
+      <c r="W12" s="5"/>
+      <c r="X12" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y12" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z12" s="5"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="6"/>
-      <c r="X13" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y13" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z13" s="6"/>
+      <c r="B13" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
+      <c r="V13" s="5"/>
+      <c r="W13" s="5"/>
+      <c r="X13" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y13" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z13" s="5"/>
     </row>
     <row r="14" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="6"/>
-      <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
-      <c r="V14" s="6"/>
-      <c r="W14" s="6"/>
-      <c r="X14" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y14" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z14" s="6"/>
+      <c r="B14" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="5"/>
+      <c r="U14" s="5"/>
+      <c r="V14" s="5"/>
+      <c r="W14" s="5"/>
+      <c r="X14" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y14" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z14" s="5"/>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
-      <c r="T15" s="6"/>
-      <c r="U15" s="6"/>
-      <c r="V15" s="6"/>
-      <c r="W15" s="6"/>
-      <c r="X15" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y15" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z15" s="6"/>
+      <c r="B15" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="5"/>
+      <c r="U15" s="5"/>
+      <c r="V15" s="5"/>
+      <c r="W15" s="5"/>
+      <c r="X15" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y15" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z15" s="5"/>
     </row>
     <row r="16" spans="1:26" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Q16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="R16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="S16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="T16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="U16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="V16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="W16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="X16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y16" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z16" s="6"/>
+      <c r="B16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="P16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="R16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="S16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="T16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="U16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="V16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="W16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="X16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y16" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z16" s="5"/>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="L17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="N17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="O17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="P17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Q17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="R17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="S17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="T17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="U17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="V17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="W17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="X17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Y17" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Z17" s="6"/>
+      <c r="B17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="P17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="S17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="T17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="U17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="V17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="W17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="X17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Y17" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z17" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6743,6 +6780,12 @@
       <c r="C10" s="3" t="s">
         <v>430</v>
       </c>
+      <c r="D10" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>416</v>
+      </c>
       <c r="X10" s="3" t="s">
         <v>430</v>
       </c>

</xml_diff>

<commit_message>
added new fluoro handles
</commit_message>
<xml_diff>
--- a/crisscross_kit/crisscross/dna_source_plates/assembly_plates/sw_src011_fluorescenthandles.xlsx
+++ b/crisscross_kit/crisscross/dna_source_plates/assembly_plates/sw_src011_fluorescenthandles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stellawang/Documents/gitrepos/Crisscross-Design/crisscross_kit/crisscross/dna_source_plates/assembly_plates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt/Documents/Shih_Lab_Postdoc/research_projects/crisscross_code/crisscross_kit/crisscross/dna_source_plates/assembly_plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA305B96-40A4-3E40-98BC-0F92CB9BEA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FFB62C7-142F-0C4A-ABCB-0CF25F721A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="25600" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="467">
   <si>
     <t>well</t>
   </si>
@@ -1384,6 +1384,45 @@
   </si>
   <si>
     <t>TATTTATCCCAAGCATTAGACGGGAGAATTATAAGAGCAAGAtt TCCACTA /3ATTO647N/</t>
+  </si>
+  <si>
+    <t>ASSEMBLY-FLUOR488-MAD-33-h5-position_3</t>
+  </si>
+  <si>
+    <t>ASSEMBLY-FLUOR488-MAD-19-h5-position_14</t>
+  </si>
+  <si>
+    <t>ASSEMBLY-FLUOR488-MAD-54-h5-position_26</t>
+  </si>
+  <si>
+    <t>ASSEMBLY_HANDLE_v2-33-h5-position_3</t>
+  </si>
+  <si>
+    <t>TCTGTGGTGGCTCACAATTCCACACAACCGGTCACGCTGCGCttCGTAGAT/3ATTO488N/</t>
+  </si>
+  <si>
+    <t>Fluorescent Assembly Handle For Slat Position 3, Handle 33, Fluorophore Atto488 Side h5, MAD</t>
+  </si>
+  <si>
+    <t>atto488n</t>
+  </si>
+  <si>
+    <t>ASSEMBLY_HANDLE_v2-19-h5-position_14</t>
+  </si>
+  <si>
+    <t>GATAAAAACGGTCTTTACCCTGACTATTTGGCCAACAGAGATttGGATCTT/3ATTO488N/</t>
+  </si>
+  <si>
+    <t>Fluorescent Assembly Handle For Slat Position 14, Handle 19, Fluorophore Atto488 Side h5,MAD</t>
+  </si>
+  <si>
+    <t>ASSEMBLY_HANDLE_v2-54-h5-position_26</t>
+  </si>
+  <si>
+    <t>CTTTACAGAGAAGCCCTTTTTAAGAAAACCAGAAGGAGCGGAttGGACTTA/3ATTO488N/</t>
+  </si>
+  <si>
+    <t>Fluorescent Assembly Handle For Slat Position 26, Handle 54, Fluorophore Atto488 Side h5, MAD</t>
   </si>
 </sst>
 </file>
@@ -3004,7 +3043,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>100</v>
       </c>
@@ -3021,7 +3060,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>101</v>
       </c>
@@ -3038,7 +3077,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>102</v>
       </c>
@@ -3055,67 +3094,112 @@
         <v>100</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B100" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="C100" t="s">
+        <v>458</v>
+      </c>
+      <c r="D100" t="s">
+        <v>459</v>
+      </c>
+      <c r="E100">
+        <v>100</v>
+      </c>
+      <c r="F100" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B101" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="C101" t="s">
+        <v>462</v>
+      </c>
+      <c r="D101" t="s">
+        <v>463</v>
+      </c>
+      <c r="E101">
+        <v>100</v>
+      </c>
+      <c r="F101" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B102" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C102" t="s">
+        <v>465</v>
+      </c>
+      <c r="D102" t="s">
+        <v>466</v>
+      </c>
+      <c r="E102">
+        <v>100</v>
+      </c>
+      <c r="F102" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>115</v>
       </c>
@@ -5884,9 +5968,15 @@
       <c r="C6" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="D6" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>456</v>
+      </c>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -6712,6 +6802,15 @@
       <c r="C6" s="3" t="s">
         <v>430</v>
       </c>
+      <c r="D6" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>416</v>
+      </c>
       <c r="X6" s="3" t="s">
         <v>430</v>
       </c>

</xml_diff>